<commit_message>
Fix copyright year UI
</commit_message>
<xml_diff>
--- a/Chatly_Proyeksi_Keuangan.xlsx
+++ b/Chatly_Proyeksi_Keuangan.xlsx
@@ -974,7 +974,7 @@
         </is>
       </c>
       <c r="C5" s="16" t="n">
-        <v>16000</v>
+        <v>18000</v>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
@@ -1224,11 +1224,11 @@
         </is>
       </c>
       <c r="C28" s="18" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>basis dari beta / early sales</t>
+          <t>basis dari beta / early sales (konservatif)</t>
         </is>
       </c>
     </row>
@@ -1239,11 +1239,11 @@
         </is>
       </c>
       <c r="C29" s="18" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t>ramp linear</t>
+          <t>ramp linear (konservatif)</t>
         </is>
       </c>
     </row>
@@ -1254,11 +1254,11 @@
         </is>
       </c>
       <c r="C30" s="18" t="n">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t>ramp linear seiring tim sales &amp; marketing</t>
+          <t>ramp linear (konservatif)</t>
         </is>
       </c>
     </row>
@@ -1269,11 +1269,11 @@
         </is>
       </c>
       <c r="C31" s="19" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t>% pelanggan berhenti / bln (SMB SaaS)</t>
+          <t>% pelanggan berhenti / bln (SMB SaaS, konservatif)</t>
         </is>
       </c>
     </row>
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="C32" s="19" t="n">
-        <v>0.4</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="33">
@@ -1294,7 +1294,7 @@
         </is>
       </c>
       <c r="C33" s="19" t="n">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="34">
@@ -1304,7 +1304,7 @@
         </is>
       </c>
       <c r="C34" s="19" t="n">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="35">
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="C39" s="16" t="n">
-        <v>18000000</v>
+        <v>3500000</v>
       </c>
       <c r="D39" s="18" t="n">
         <v>1</v>
@@ -1370,7 +1370,7 @@
         </is>
       </c>
       <c r="C40" s="16" t="n">
-        <v>18000000</v>
+        <v>3500000</v>
       </c>
       <c r="D40" s="18" t="n">
         <v>1</v>
@@ -1383,7 +1383,7 @@
         </is>
       </c>
       <c r="C41" s="16" t="n">
-        <v>13000000</v>
+        <v>3500000</v>
       </c>
       <c r="D41" s="18" t="n">
         <v>1</v>
@@ -1396,7 +1396,7 @@
         </is>
       </c>
       <c r="C42" s="16" t="n">
-        <v>9000000</v>
+        <v>2500000</v>
       </c>
       <c r="D42" s="18" t="n">
         <v>1</v>
@@ -1409,10 +1409,10 @@
         </is>
       </c>
       <c r="C43" s="16" t="n">
-        <v>12000000</v>
+        <v>3000000</v>
       </c>
       <c r="D43" s="18" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
@@ -1422,10 +1422,10 @@
         </is>
       </c>
       <c r="C44" s="16" t="n">
-        <v>7000000</v>
+        <v>2000000</v>
       </c>
       <c r="D44" s="18" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -1435,10 +1435,10 @@
         </is>
       </c>
       <c r="C45" s="16" t="n">
-        <v>15000000</v>
+        <v>3500000</v>
       </c>
       <c r="D45" s="18" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -1448,10 +1448,10 @@
         </is>
       </c>
       <c r="C46" s="16" t="n">
-        <v>9000000</v>
+        <v>2500000</v>
       </c>
       <c r="D46" s="18" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -1525,14 +1525,14 @@
     <row r="53">
       <c r="B53" t="inlineStr">
         <is>
-          <t>Kantor &amp; Admin</t>
+          <t>Operasional &amp; Admin</t>
         </is>
       </c>
       <c r="C53" s="16" t="n">
-        <v>5000000</v>
+        <v>1500000</v>
       </c>
       <c r="D53" s="16" t="n">
-        <v>10000000</v>
+        <v>3000000</v>
       </c>
     </row>
     <row r="54">
@@ -1542,10 +1542,10 @@
         </is>
       </c>
       <c r="C54" s="16" t="n">
-        <v>10000000</v>
+        <v>8000000</v>
       </c>
       <c r="D54" s="16" t="n">
-        <v>40000000</v>
+        <v>25000000</v>
       </c>
     </row>
     <row r="56">
@@ -5547,7 +5547,7 @@
     <row r="31">
       <c r="B31" t="inlineStr">
         <is>
-          <t>OPEX - Kantor &amp; Admin</t>
+          <t>OPEX - Operasional &amp; Admin</t>
         </is>
       </c>
       <c r="C31" s="6">

</xml_diff>